<commit_message>
2023-06-29   Lambda  sku 对照表开发
</commit_message>
<xml_diff>
--- a/erp-server/erp-server-oms/src/main/resources/excel/skuMaping.xlsx
+++ b/erp-server/erp-server-oms/src/main/resources/excel/skuMaping.xlsx
@@ -243,7 +243,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -261,6 +261,15 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -567,8 +576,9 @@
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="27.875" customWidth="1"/>
-    <col min="2" max="4" width="20.5" customWidth="1"/>
-    <col min="5" max="5" width="32.625" customWidth="1"/>
+    <col min="2" max="2" width="20.5" customWidth="1"/>
+    <col min="3" max="4" width="20.5" style="7" customWidth="1"/>
+    <col min="5" max="5" width="32.625" style="7" customWidth="1"/>
     <col min="6" max="6" width="21.75" customWidth="1"/>
     <col min="7" max="7" width="19.125" customWidth="1"/>
     <col min="8" max="8" width="22" customWidth="1"/>
@@ -582,13 +592,13 @@
       <c r="B1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="8" t="s">
         <v>0</v>
       </c>
       <c r="F1" s="3" t="s">
@@ -611,13 +621,13 @@
       <c r="B2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="6" t="s">
         <v>9</v>
       </c>
       <c r="F2" s="2" t="s">

</xml_diff>